<commit_message>
Daily NAV update 2026-03-12
</commit_message>
<xml_diff>
--- a/output/nav_changes_2026-03-12.xlsx
+++ b/output/nav_changes_2026-03-12.xlsx
@@ -92,8 +92,8 @@
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="10" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="10" fontId="2" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" wrapText="1"/>
@@ -551,18 +551,16 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>TMX:DYN27550</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
+          <t>2026-03-11</t>
+        </is>
+      </c>
+      <c r="D3" s="5" t="n">
+        <v>15.95</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
@@ -605,7 +603,7 @@
       <c r="F4" s="3" t="n">
         <v>-0.04</v>
       </c>
-      <c r="G4" s="5" t="n">
+      <c r="G4" s="6" t="n">
         <v>-0.001989</v>
       </c>
     </row>
@@ -625,28 +623,28 @@
           <t>2026-03-11</t>
         </is>
       </c>
-      <c r="D5" s="6" t="n">
+      <c r="D5" s="5" t="n">
         <v>21.48</v>
       </c>
-      <c r="E5" s="6" t="n">
+      <c r="E5" s="5" t="n">
         <v>21.58</v>
       </c>
-      <c r="F5" s="6" t="n">
+      <c r="F5" s="5" t="n">
         <v>-0.1</v>
       </c>
-      <c r="G5" s="5" t="n">
+      <c r="G5" s="6" t="n">
         <v>-0.004634</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>XIG US IG Corp Bond (CAD Hdg)</t>
+          <t>Lysander-Canso Corp Value Bond F</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>XIG.TO</t>
+          <t>0P0000XXNG.TO</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
@@ -655,27 +653,27 @@
         </is>
       </c>
       <c r="D6" s="3" t="n">
-        <v>19.61</v>
+        <v>14.0873</v>
       </c>
       <c r="E6" s="3" t="n">
-        <v>19.76</v>
+        <v>14.1399</v>
       </c>
       <c r="F6" s="3" t="n">
-        <v>-0.15</v>
-      </c>
-      <c r="G6" s="5" t="n">
-        <v>-0.007591</v>
+        <v>-0.0526</v>
+      </c>
+      <c r="G6" s="6" t="n">
+        <v>-0.00372</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>XCB Cdn Corporate Bond</t>
+          <t>Lysander-Fulcra Corp Sec F</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>XCB.TO</t>
+          <t>0P0001CIH7.TO</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -683,28 +681,28 @@
           <t>2026-03-11</t>
         </is>
       </c>
-      <c r="D7" s="6" t="n">
-        <v>20.1</v>
-      </c>
-      <c r="E7" s="6" t="n">
-        <v>20.21</v>
-      </c>
-      <c r="F7" s="6" t="n">
-        <v>-0.11</v>
-      </c>
-      <c r="G7" s="5" t="n">
-        <v>-0.005443</v>
+      <c r="D7" s="5" t="n">
+        <v>9.513999999999999</v>
+      </c>
+      <c r="E7" s="5" t="n">
+        <v>9.524900000000001</v>
+      </c>
+      <c r="F7" s="5" t="n">
+        <v>-0.0109</v>
+      </c>
+      <c r="G7" s="6" t="n">
+        <v>-0.001144</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>PIMCO Monthly Income F</t>
+          <t>Pender Corporate Bond F</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>PMIF.TO</t>
+          <t>0P0000MOQB.TO</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
@@ -713,27 +711,27 @@
         </is>
       </c>
       <c r="D8" s="3" t="n">
-        <v>18.235</v>
+        <v>14.2898</v>
       </c>
       <c r="E8" s="3" t="n">
-        <v>18.27</v>
+        <v>14.3083</v>
       </c>
       <c r="F8" s="3" t="n">
-        <v>-0.035</v>
-      </c>
-      <c r="G8" s="5" t="n">
-        <v>-0.001916</v>
+        <v>-0.0185</v>
+      </c>
+      <c r="G8" s="6" t="n">
+        <v>-0.001293</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Manulife Strategic Income F</t>
+          <t>XIG US IG Corp Bond (CAD Hdg)</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>0P0000NFNA.TO</t>
+          <t>XIG.TO</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -741,28 +739,28 @@
           <t>2026-03-11</t>
         </is>
       </c>
-      <c r="D9" s="6" t="n">
-        <v>11.2193</v>
-      </c>
-      <c r="E9" s="6" t="n">
-        <v>11.245</v>
-      </c>
-      <c r="F9" s="6" t="n">
-        <v>-0.0257</v>
-      </c>
-      <c r="G9" s="5" t="n">
-        <v>-0.002285</v>
+      <c r="D9" s="5" t="n">
+        <v>19.61</v>
+      </c>
+      <c r="E9" s="5" t="n">
+        <v>19.76</v>
+      </c>
+      <c r="F9" s="5" t="n">
+        <v>-0.15</v>
+      </c>
+      <c r="G9" s="6" t="n">
+        <v>-0.007591</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>Lysander-Canso Corp Value Bond F</t>
+          <t>XCB Cdn Corporate Bond</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>0P0000XXNG.TO</t>
+          <t>XCB.TO</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
@@ -771,27 +769,27 @@
         </is>
       </c>
       <c r="D10" s="3" t="n">
-        <v>14.0873</v>
+        <v>20.1</v>
       </c>
       <c r="E10" s="3" t="n">
-        <v>14.1399</v>
+        <v>20.21</v>
       </c>
       <c r="F10" s="3" t="n">
-        <v>-0.0526</v>
-      </c>
-      <c r="G10" s="5" t="n">
-        <v>-0.00372</v>
+        <v>-0.11</v>
+      </c>
+      <c r="G10" s="6" t="n">
+        <v>-0.005443</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Pender Corporate Bond F</t>
+          <t>PIMCO Monthly Income F</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>0P0000MOQB.TO</t>
+          <t>PMIF.TO</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -799,28 +797,28 @@
           <t>2026-03-11</t>
         </is>
       </c>
-      <c r="D11" s="6" t="n">
-        <v>14.2898</v>
-      </c>
-      <c r="E11" s="6" t="n">
-        <v>14.3083</v>
-      </c>
-      <c r="F11" s="6" t="n">
-        <v>-0.0185</v>
-      </c>
-      <c r="G11" s="5" t="n">
-        <v>-0.001293</v>
+      <c r="D11" s="5" t="n">
+        <v>18.235</v>
+      </c>
+      <c r="E11" s="5" t="n">
+        <v>18.27</v>
+      </c>
+      <c r="F11" s="5" t="n">
+        <v>-0.035</v>
+      </c>
+      <c r="G11" s="6" t="n">
+        <v>-0.001916</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>Lysander-Fulcra Corp Sec F</t>
+          <t>Manulife Strategic Income F</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>0P0001CIH7.TO</t>
+          <t>0P0000NFNA.TO</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
@@ -829,16 +827,16 @@
         </is>
       </c>
       <c r="D12" s="3" t="n">
-        <v>9.513999999999999</v>
+        <v>11.2193</v>
       </c>
       <c r="E12" s="3" t="n">
-        <v>9.524900000000001</v>
+        <v>11.245</v>
       </c>
       <c r="F12" s="3" t="n">
-        <v>-0.0109</v>
-      </c>
-      <c r="G12" s="5" t="n">
-        <v>-0.001144</v>
+        <v>-0.0257</v>
+      </c>
+      <c r="G12" s="6" t="n">
+        <v>-0.002285</v>
       </c>
     </row>
     <row r="13">
@@ -857,16 +855,16 @@
           <t>2026-03-11</t>
         </is>
       </c>
-      <c r="D13" s="6" t="n">
+      <c r="D13" s="5" t="n">
         <v>9.1845</v>
       </c>
-      <c r="E13" s="6" t="n">
+      <c r="E13" s="5" t="n">
         <v>9.2263</v>
       </c>
-      <c r="F13" s="6" t="n">
+      <c r="F13" s="5" t="n">
         <v>-0.0418</v>
       </c>
-      <c r="G13" s="5" t="n">
+      <c r="G13" s="6" t="n">
         <v>-0.004531</v>
       </c>
     </row>
@@ -895,7 +893,7 @@
       <c r="F14" s="3" t="n">
         <v>-0.0241</v>
       </c>
-      <c r="G14" s="5" t="n">
+      <c r="G14" s="6" t="n">
         <v>-0.002736</v>
       </c>
     </row>
@@ -915,16 +913,16 @@
           <t>2026-03-11</t>
         </is>
       </c>
-      <c r="D15" s="6" t="n">
+      <c r="D15" s="5" t="n">
         <v>9.793100000000001</v>
       </c>
-      <c r="E15" s="6" t="n">
+      <c r="E15" s="5" t="n">
         <v>9.8253</v>
       </c>
-      <c r="F15" s="6" t="n">
+      <c r="F15" s="5" t="n">
         <v>-0.0322</v>
       </c>
-      <c r="G15" s="5" t="n">
+      <c r="G15" s="6" t="n">
         <v>-0.003277</v>
       </c>
     </row>
@@ -939,7 +937,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N42"/>
+  <dimension ref="A1:O42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -956,6 +954,7 @@
     <col width="20" customWidth="1" min="12" max="12"/>
     <col width="20" customWidth="1" min="13" max="13"/>
     <col width="20" customWidth="1" min="14" max="14"/>
+    <col width="20" customWidth="1" min="15" max="15"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -971,62 +970,67 @@
       </c>
       <c r="C1" s="8" t="inlineStr">
         <is>
+          <t>Dynamic Short Term Credit PLUS F</t>
+        </is>
+      </c>
+      <c r="D1" s="8" t="inlineStr">
+        <is>
+          <t>DXDB Dynamic Discount Bond ETF</t>
+        </is>
+      </c>
+      <c r="E1" s="8" t="inlineStr">
+        <is>
+          <t>Lysander-Canso Corp Value Bond F</t>
+        </is>
+      </c>
+      <c r="F1" s="8" t="inlineStr">
+        <is>
+          <t>Lysander-Fulcra Corp Sec F</t>
+        </is>
+      </c>
+      <c r="G1" s="8" t="inlineStr">
+        <is>
+          <t>Pender Corporate Bond F</t>
+        </is>
+      </c>
+      <c r="H1" s="8" t="inlineStr">
+        <is>
+          <t>XIG US IG Corp Bond (CAD Hdg)</t>
+        </is>
+      </c>
+      <c r="I1" s="8" t="inlineStr">
+        <is>
+          <t>XCB Cdn Corporate Bond</t>
+        </is>
+      </c>
+      <c r="J1" s="8" t="inlineStr">
+        <is>
+          <t>PIMCO Monthly Income F</t>
+        </is>
+      </c>
+      <c r="K1" s="8" t="inlineStr">
+        <is>
           <t>Manulife Strategic Income F</t>
         </is>
       </c>
-      <c r="D1" s="8" t="inlineStr">
-        <is>
-          <t>Lysander-Canso Corp Value Bond F</t>
-        </is>
-      </c>
-      <c r="E1" s="8" t="inlineStr">
-        <is>
-          <t>PIMCO Monthly Income F</t>
-        </is>
-      </c>
-      <c r="F1" s="8" t="inlineStr">
+      <c r="L1" s="8" t="inlineStr">
         <is>
           <t>RBC Global Bond F</t>
         </is>
       </c>
-      <c r="G1" s="8" t="inlineStr">
+      <c r="M1" s="8" t="inlineStr">
         <is>
           <t>Mackenzie Unconstrained FI F</t>
         </is>
       </c>
-      <c r="H1" s="8" t="inlineStr">
-        <is>
-          <t>XIG US IG Corp Bond (CAD Hdg)</t>
-        </is>
-      </c>
-      <c r="I1" s="8" t="inlineStr">
-        <is>
-          <t>XCB Cdn Corporate Bond</t>
-        </is>
-      </c>
-      <c r="J1" s="8" t="inlineStr">
-        <is>
-          <t>DXDB Dynamic Discount Bond ETF</t>
-        </is>
-      </c>
-      <c r="K1" s="8" t="inlineStr">
-        <is>
-          <t>Lysander-Fulcra Corp Sec F</t>
-        </is>
-      </c>
-      <c r="L1" s="8" t="inlineStr">
+      <c r="N1" s="8" t="inlineStr">
         <is>
           <t>RBC Core Bond F</t>
         </is>
       </c>
-      <c r="M1" s="8" t="inlineStr">
-        <is>
-          <t>Dynamic Short Term Credit PLUS F</t>
-        </is>
-      </c>
-      <c r="N1" s="8" t="inlineStr">
-        <is>
-          <t>Pender Corporate Bond F</t>
+      <c r="O1" s="8" t="inlineStr">
+        <is>
+          <t>Dynamic Credit Abs Return F</t>
         </is>
       </c>
     </row>
@@ -1039,42 +1043,43 @@
       <c r="B2" s="9" t="n">
         <v>0</v>
       </c>
-      <c r="C2" s="5" t="n">
+      <c r="C2" s="6" t="n">
+        <v>-0.001989</v>
+      </c>
+      <c r="D2" s="6" t="n">
+        <v>-0.004634</v>
+      </c>
+      <c r="E2" s="6" t="n">
+        <v>-0.00372</v>
+      </c>
+      <c r="F2" s="6" t="n">
+        <v>-0.001144</v>
+      </c>
+      <c r="G2" s="6" t="n">
+        <v>-0.001293</v>
+      </c>
+      <c r="H2" s="6" t="n">
+        <v>-0.007591</v>
+      </c>
+      <c r="I2" s="6" t="n">
+        <v>-0.005443</v>
+      </c>
+      <c r="J2" s="6" t="n">
+        <v>-0.001916</v>
+      </c>
+      <c r="K2" s="6" t="n">
         <v>-0.002285</v>
       </c>
-      <c r="D2" s="5" t="n">
-        <v>-0.00372</v>
-      </c>
-      <c r="E2" s="5" t="n">
-        <v>-0.001916</v>
-      </c>
-      <c r="F2" s="5" t="n">
+      <c r="L2" s="6" t="n">
         <v>-0.004531</v>
       </c>
-      <c r="G2" s="5" t="n">
+      <c r="M2" s="6" t="n">
         <v>-0.002736</v>
       </c>
-      <c r="H2" s="5" t="n">
-        <v>-0.007591</v>
-      </c>
-      <c r="I2" s="5" t="n">
-        <v>-0.005443</v>
-      </c>
-      <c r="J2" s="5" t="n">
-        <v>-0.004634</v>
-      </c>
-      <c r="K2" s="5" t="n">
-        <v>-0.001144</v>
-      </c>
-      <c r="L2" s="5" t="n">
+      <c r="N2" s="6" t="n">
         <v>-0.003277</v>
       </c>
-      <c r="M2" s="5" t="n">
-        <v>-0.001989</v>
-      </c>
-      <c r="N2" s="5" t="n">
-        <v>-0.001293</v>
-      </c>
+      <c r="O2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -1085,42 +1090,43 @@
       <c r="B3" s="9" t="n">
         <v>0</v>
       </c>
-      <c r="C3" s="10" t="n">
+      <c r="C3" s="6" t="n">
+        <v>-0.00149</v>
+      </c>
+      <c r="D3" s="6" t="n">
+        <v>-0.00185</v>
+      </c>
+      <c r="E3" s="6" t="n">
+        <v>-0.000382</v>
+      </c>
+      <c r="F3" s="10" t="n">
+        <v>0.000378</v>
+      </c>
+      <c r="G3" s="10" t="n">
+        <v>0.000804</v>
+      </c>
+      <c r="H3" s="6" t="n">
+        <v>-0.005536</v>
+      </c>
+      <c r="I3" s="6" t="n">
+        <v>-0.000495</v>
+      </c>
+      <c r="J3" s="10" t="n">
+        <v>0.000274</v>
+      </c>
+      <c r="K3" s="10" t="n">
         <v>0.001657</v>
       </c>
-      <c r="D3" s="5" t="n">
-        <v>-0.000382</v>
-      </c>
-      <c r="E3" s="10" t="n">
-        <v>0.000274</v>
-      </c>
-      <c r="F3" s="10" t="n">
+      <c r="L3" s="10" t="n">
         <v>0.001172</v>
       </c>
-      <c r="G3" s="10" t="n">
+      <c r="M3" s="10" t="n">
         <v>0.000102</v>
       </c>
-      <c r="H3" s="5" t="n">
-        <v>-0.005536</v>
-      </c>
-      <c r="I3" s="5" t="n">
-        <v>-0.000495</v>
-      </c>
-      <c r="J3" s="5" t="n">
-        <v>-0.00185</v>
-      </c>
-      <c r="K3" s="10" t="n">
-        <v>0.000378</v>
-      </c>
-      <c r="L3" s="10" t="n">
+      <c r="N3" s="10" t="n">
         <v>0.000285</v>
       </c>
-      <c r="M3" s="5" t="n">
-        <v>-0.00149</v>
-      </c>
-      <c r="N3" s="10" t="n">
-        <v>0.000804</v>
-      </c>
+      <c r="O3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -1128,23 +1134,23 @@
           <t>2026-03-09</t>
         </is>
       </c>
-      <c r="B4" s="5" t="n">
+      <c r="B4" s="6" t="n">
         <v>-0.002505</v>
       </c>
-      <c r="C4" s="5" t="n">
-        <v>-0.001991</v>
+      <c r="C4" s="6" t="n">
+        <v>-0.000992</v>
       </c>
       <c r="D4" s="10" t="n">
+        <v>0.001854</v>
+      </c>
+      <c r="E4" s="10" t="n">
         <v>0.001388</v>
       </c>
-      <c r="E4" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="F4" s="10" t="n">
-        <v>0.000369</v>
-      </c>
-      <c r="G4" s="5" t="n">
-        <v>-0.000499</v>
+      <c r="F4" s="6" t="n">
+        <v>-0.001102</v>
+      </c>
+      <c r="G4" s="10" t="n">
+        <v>0.002665</v>
       </c>
       <c r="H4" s="10" t="n">
         <v>0.005058</v>
@@ -1152,21 +1158,22 @@
       <c r="I4" s="10" t="n">
         <v>0.001982</v>
       </c>
-      <c r="J4" s="10" t="n">
-        <v>0.001854</v>
-      </c>
-      <c r="K4" s="5" t="n">
-        <v>-0.001102</v>
+      <c r="J4" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="K4" s="6" t="n">
+        <v>-0.001991</v>
       </c>
       <c r="L4" s="10" t="n">
+        <v>0.000369</v>
+      </c>
+      <c r="M4" s="6" t="n">
+        <v>-0.000499</v>
+      </c>
+      <c r="N4" s="10" t="n">
         <v>0.0009779999999999999</v>
       </c>
-      <c r="M4" s="5" t="n">
-        <v>-0.000992</v>
-      </c>
-      <c r="N4" s="10" t="n">
-        <v>0.002665</v>
-      </c>
+      <c r="O4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -1177,42 +1184,43 @@
       <c r="B5" s="9" t="n">
         <v>0</v>
       </c>
-      <c r="C5" s="5" t="n">
+      <c r="C5" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="D5" s="6" t="n">
+        <v>-0.002773</v>
+      </c>
+      <c r="E5" s="6" t="n">
+        <v>-0.003548</v>
+      </c>
+      <c r="F5" s="6" t="n">
+        <v>-0.003356</v>
+      </c>
+      <c r="G5" s="6" t="n">
+        <v>-0.001785</v>
+      </c>
+      <c r="H5" s="6" t="n">
+        <v>-0.004030000000000001</v>
+      </c>
+      <c r="I5" s="6" t="n">
+        <v>-0.003457</v>
+      </c>
+      <c r="J5" s="6" t="n">
+        <v>-0.003274</v>
+      </c>
+      <c r="K5" s="6" t="n">
         <v>-0.003561</v>
       </c>
-      <c r="D5" s="5" t="n">
-        <v>-0.003548</v>
-      </c>
-      <c r="E5" s="5" t="n">
-        <v>-0.003274</v>
-      </c>
-      <c r="F5" s="5" t="n">
+      <c r="L5" s="6" t="n">
         <v>-0.002123</v>
       </c>
-      <c r="G5" s="5" t="n">
+      <c r="M5" s="6" t="n">
         <v>-0.001462</v>
       </c>
-      <c r="H5" s="5" t="n">
-        <v>-0.004030000000000001</v>
-      </c>
-      <c r="I5" s="5" t="n">
-        <v>-0.003457</v>
-      </c>
-      <c r="J5" s="5" t="n">
-        <v>-0.002773</v>
-      </c>
-      <c r="K5" s="5" t="n">
-        <v>-0.003356</v>
-      </c>
-      <c r="L5" s="5" t="n">
+      <c r="N5" s="6" t="n">
         <v>-0.002977</v>
       </c>
-      <c r="M5" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="N5" s="5" t="n">
-        <v>-0.001785</v>
-      </c>
+      <c r="O5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -1223,42 +1231,43 @@
       <c r="B6" s="10" t="n">
         <v>0.000501</v>
       </c>
-      <c r="C6" s="5" t="n">
+      <c r="C6" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="D6" s="6" t="n">
+        <v>-0.003683</v>
+      </c>
+      <c r="E6" s="6" t="n">
+        <v>-0.003648</v>
+      </c>
+      <c r="F6" s="6" t="n">
+        <v>-0.002056</v>
+      </c>
+      <c r="G6" s="6" t="n">
+        <v>-0.005763000000000001</v>
+      </c>
+      <c r="H6" s="6" t="n">
+        <v>-0.003514</v>
+      </c>
+      <c r="I6" s="6" t="n">
+        <v>-0.004425</v>
+      </c>
+      <c r="J6" s="6" t="n">
+        <v>-0.000273</v>
+      </c>
+      <c r="K6" s="6" t="n">
         <v>-0.002536</v>
       </c>
-      <c r="D6" s="5" t="n">
-        <v>-0.003648</v>
-      </c>
-      <c r="E6" s="5" t="n">
-        <v>-0.000273</v>
-      </c>
-      <c r="F6" s="5" t="n">
+      <c r="L6" s="6" t="n">
         <v>-0.003766</v>
       </c>
-      <c r="G6" s="5" t="n">
+      <c r="M6" s="6" t="n">
         <v>-0.00172</v>
       </c>
-      <c r="H6" s="5" t="n">
-        <v>-0.003514</v>
-      </c>
-      <c r="I6" s="5" t="n">
-        <v>-0.004425</v>
-      </c>
-      <c r="J6" s="5" t="n">
-        <v>-0.003683</v>
-      </c>
-      <c r="K6" s="5" t="n">
-        <v>-0.002056</v>
-      </c>
-      <c r="L6" s="5" t="n">
+      <c r="N6" s="6" t="n">
         <v>-0.002675</v>
       </c>
-      <c r="M6" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="N6" s="5" t="n">
-        <v>-0.005763000000000001</v>
-      </c>
+      <c r="O6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -1266,23 +1275,23 @@
           <t>2026-03-04</t>
         </is>
       </c>
-      <c r="B7" s="5" t="n">
+      <c r="B7" s="6" t="n">
         <v>-0.0025</v>
       </c>
       <c r="C7" s="10" t="n">
-        <v>0.001008</v>
-      </c>
-      <c r="D7" s="5" t="n">
+        <v>0.000993</v>
+      </c>
+      <c r="D7" s="10" t="n">
+        <v>0.0009220000000000001</v>
+      </c>
+      <c r="E7" s="6" t="n">
         <v>-0.000169</v>
       </c>
-      <c r="E7" s="5" t="n">
-        <v>-0.002177</v>
-      </c>
       <c r="F7" s="10" t="n">
-        <v>0.000443</v>
+        <v>0.001065</v>
       </c>
       <c r="G7" s="10" t="n">
-        <v>6.8e-05</v>
+        <v>0.002827</v>
       </c>
       <c r="H7" s="10" t="n">
         <v>0.001005</v>
@@ -1290,21 +1299,22 @@
       <c r="I7" s="10" t="n">
         <v>0.0009840000000000001</v>
       </c>
-      <c r="J7" s="10" t="n">
-        <v>0.0009220000000000001</v>
+      <c r="J7" s="6" t="n">
+        <v>-0.002177</v>
       </c>
       <c r="K7" s="10" t="n">
-        <v>0.001065</v>
+        <v>0.001008</v>
       </c>
       <c r="L7" s="10" t="n">
+        <v>0.000443</v>
+      </c>
+      <c r="M7" s="10" t="n">
+        <v>6.8e-05</v>
+      </c>
+      <c r="N7" s="10" t="n">
         <v>0.0005369999999999999</v>
       </c>
-      <c r="M7" s="10" t="n">
-        <v>0.000993</v>
-      </c>
-      <c r="N7" s="10" t="n">
-        <v>0.002827</v>
-      </c>
+      <c r="O7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -1312,45 +1322,46 @@
           <t>2026-03-03</t>
         </is>
       </c>
-      <c r="B8" s="5" t="n">
+      <c r="B8" s="6" t="n">
         <v>-0.001498</v>
       </c>
-      <c r="C8" s="5" t="n">
+      <c r="C8" s="6" t="n">
+        <v>-0.002476</v>
+      </c>
+      <c r="D8" s="6" t="n">
+        <v>-0.001381</v>
+      </c>
+      <c r="E8" s="6" t="n">
+        <v>-0.001943</v>
+      </c>
+      <c r="F8" s="6" t="n">
+        <v>-0.005051</v>
+      </c>
+      <c r="G8" s="6" t="n">
+        <v>-0.009876000000000001</v>
+      </c>
+      <c r="H8" s="6" t="n">
+        <v>-0.0005020000000000001</v>
+      </c>
+      <c r="I8" s="6" t="n">
+        <v>-0.001474</v>
+      </c>
+      <c r="J8" s="6" t="n">
+        <v>-0.003256</v>
+      </c>
+      <c r="K8" s="6" t="n">
         <v>-0.004026</v>
       </c>
-      <c r="D8" s="5" t="n">
-        <v>-0.001943</v>
-      </c>
-      <c r="E8" s="5" t="n">
-        <v>-0.003256</v>
-      </c>
-      <c r="F8" s="5" t="n">
+      <c r="L8" s="6" t="n">
         <v>-0.003679</v>
       </c>
-      <c r="G8" s="5" t="n">
+      <c r="M8" s="6" t="n">
         <v>-0.002089</v>
       </c>
-      <c r="H8" s="5" t="n">
-        <v>-0.0005020000000000001</v>
-      </c>
-      <c r="I8" s="5" t="n">
-        <v>-0.001474</v>
-      </c>
-      <c r="J8" s="5" t="n">
-        <v>-0.001381</v>
-      </c>
-      <c r="K8" s="5" t="n">
-        <v>-0.005051</v>
-      </c>
-      <c r="L8" s="5" t="n">
+      <c r="N8" s="6" t="n">
         <v>-0.002377</v>
       </c>
-      <c r="M8" s="5" t="n">
-        <v>-0.002476</v>
-      </c>
-      <c r="N8" s="5" t="n">
-        <v>-0.009876000000000001</v>
-      </c>
+      <c r="O8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -1358,45 +1369,46 @@
           <t>2026-03-02</t>
         </is>
       </c>
-      <c r="B9" s="5" t="n">
+      <c r="B9" s="6" t="n">
         <v>-0.000499</v>
       </c>
-      <c r="C9" s="5" t="n">
+      <c r="C9" s="6" t="n">
+        <v>-0.003455</v>
+      </c>
+      <c r="D9" s="6" t="n">
+        <v>-0.003668</v>
+      </c>
+      <c r="E9" s="6" t="n">
+        <v>-0.00362</v>
+      </c>
+      <c r="F9" s="10" t="n">
+        <v>0.002396</v>
+      </c>
+      <c r="G9" s="6" t="n">
+        <v>-0.001608</v>
+      </c>
+      <c r="H9" s="6" t="n">
+        <v>-0.004002</v>
+      </c>
+      <c r="I9" s="6" t="n">
+        <v>-0.00489</v>
+      </c>
+      <c r="J9" s="6" t="n">
+        <v>-0.002166</v>
+      </c>
+      <c r="K9" s="6" t="n">
         <v>-0.002881</v>
       </c>
-      <c r="D9" s="5" t="n">
-        <v>-0.00362</v>
-      </c>
-      <c r="E9" s="5" t="n">
-        <v>-0.002166</v>
-      </c>
-      <c r="F9" s="5" t="n">
+      <c r="L9" s="6" t="n">
         <v>-0.003655</v>
       </c>
-      <c r="G9" s="5" t="n">
+      <c r="M9" s="6" t="n">
         <v>-0.002646</v>
       </c>
-      <c r="H9" s="5" t="n">
-        <v>-0.004002</v>
-      </c>
-      <c r="I9" s="5" t="n">
-        <v>-0.00489</v>
-      </c>
-      <c r="J9" s="5" t="n">
-        <v>-0.003668</v>
-      </c>
-      <c r="K9" s="10" t="n">
-        <v>0.002396</v>
-      </c>
-      <c r="L9" s="5" t="n">
+      <c r="N9" s="6" t="n">
         <v>-0.003236</v>
       </c>
-      <c r="M9" s="5" t="n">
-        <v>-0.003455</v>
-      </c>
-      <c r="N9" s="5" t="n">
-        <v>-0.001608</v>
-      </c>
+      <c r="O9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -1407,20 +1419,20 @@
       <c r="B10" s="9" t="n">
         <v>0</v>
       </c>
-      <c r="C10" s="5" t="n">
-        <v>-0.000413</v>
+      <c r="C10" s="6" t="n">
+        <v>-0.00197</v>
       </c>
       <c r="D10" s="10" t="n">
+        <v>0.000459</v>
+      </c>
+      <c r="E10" s="10" t="n">
         <v>0.000958</v>
       </c>
-      <c r="E10" s="10" t="n">
-        <v>0.00217</v>
-      </c>
       <c r="F10" s="10" t="n">
-        <v>0.000418</v>
+        <v>0.001012</v>
       </c>
       <c r="G10" s="10" t="n">
-        <v>0.000225</v>
+        <v>0.001306</v>
       </c>
       <c r="H10" s="9" t="n">
         <v>0</v>
@@ -1429,20 +1441,21 @@
         <v>0.0009790000000000001</v>
       </c>
       <c r="J10" s="10" t="n">
-        <v>0.000459</v>
-      </c>
-      <c r="K10" s="10" t="n">
-        <v>0.001012</v>
+        <v>0.00217</v>
+      </c>
+      <c r="K10" s="6" t="n">
+        <v>-0.000413</v>
       </c>
       <c r="L10" s="10" t="n">
+        <v>0.000418</v>
+      </c>
+      <c r="M10" s="10" t="n">
+        <v>0.000225</v>
+      </c>
+      <c r="N10" s="10" t="n">
         <v>5e-05</v>
       </c>
-      <c r="M10" s="5" t="n">
-        <v>-0.00197</v>
-      </c>
-      <c r="N10" s="10" t="n">
-        <v>0.001306</v>
-      </c>
+      <c r="O10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -1454,19 +1467,19 @@
         <v>0.000749</v>
       </c>
       <c r="C11" s="10" t="n">
-        <v>0.000483</v>
-      </c>
-      <c r="D11" s="5" t="n">
+        <v>0.0009859999999999999</v>
+      </c>
+      <c r="D11" s="10" t="n">
+        <v>0.0009180000000000001</v>
+      </c>
+      <c r="E11" s="6" t="n">
         <v>-0.000357</v>
       </c>
-      <c r="E11" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="F11" s="10" t="n">
-        <v>0.002752</v>
+      <c r="F11" s="6" t="n">
+        <v>-0.00099</v>
       </c>
       <c r="G11" s="10" t="n">
-        <v>1.1e-05</v>
+        <v>0.001883</v>
       </c>
       <c r="H11" s="9" t="n">
         <v>0</v>
@@ -1474,21 +1487,22 @@
       <c r="I11" s="10" t="n">
         <v>0.00049</v>
       </c>
-      <c r="J11" s="10" t="n">
-        <v>0.0009180000000000001</v>
-      </c>
-      <c r="K11" s="5" t="n">
-        <v>-0.00099</v>
+      <c r="J11" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="K11" s="10" t="n">
+        <v>0.000483</v>
       </c>
       <c r="L11" s="10" t="n">
+        <v>0.002752</v>
+      </c>
+      <c r="M11" s="10" t="n">
+        <v>1.1e-05</v>
+      </c>
+      <c r="N11" s="10" t="n">
         <v>0.0007570000000000001</v>
       </c>
-      <c r="M11" s="10" t="n">
-        <v>0.0009859999999999999</v>
-      </c>
-      <c r="N11" s="10" t="n">
-        <v>0.001883</v>
-      </c>
+      <c r="O11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1496,45 +1510,46 @@
           <t>2026-02-25</t>
         </is>
       </c>
-      <c r="B12" s="5" t="n">
+      <c r="B12" s="6" t="n">
         <v>-0.00025</v>
       </c>
-      <c r="C12" s="10" t="n">
+      <c r="C12" s="6" t="n">
+        <v>-0.000985</v>
+      </c>
+      <c r="D12" s="6" t="n">
+        <v>-0.0009170000000000001</v>
+      </c>
+      <c r="E12" s="6" t="n">
+        <v>-0.000803</v>
+      </c>
+      <c r="F12" s="10" t="n">
+        <v>0.000552</v>
+      </c>
+      <c r="G12" s="10" t="n">
+        <v>0.001324</v>
+      </c>
+      <c r="H12" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="I12" s="6" t="n">
+        <v>-0.000489</v>
+      </c>
+      <c r="J12" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="K12" s="10" t="n">
         <v>0.000105</v>
       </c>
-      <c r="D12" s="5" t="n">
-        <v>-0.000803</v>
-      </c>
-      <c r="E12" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="F12" s="5" t="n">
+      <c r="L12" s="6" t="n">
         <v>-0.0009130000000000001</v>
       </c>
-      <c r="G12" s="10" t="n">
+      <c r="M12" s="10" t="n">
         <v>7.900000000000001e-05</v>
       </c>
-      <c r="H12" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="I12" s="5" t="n">
-        <v>-0.000489</v>
-      </c>
-      <c r="J12" s="5" t="n">
-        <v>-0.0009170000000000001</v>
-      </c>
-      <c r="K12" s="10" t="n">
-        <v>0.000552</v>
-      </c>
-      <c r="L12" s="5" t="n">
+      <c r="N12" s="6" t="n">
         <v>-0.000202</v>
       </c>
-      <c r="M12" s="5" t="n">
-        <v>-0.000985</v>
-      </c>
-      <c r="N12" s="10" t="n">
-        <v>0.001324</v>
-      </c>
+      <c r="O12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -1546,41 +1561,42 @@
         <v>0.00125</v>
       </c>
       <c r="C13" s="10" t="n">
+        <v>0.000246</v>
+      </c>
+      <c r="D13" s="6" t="n">
+        <v>-0.000229</v>
+      </c>
+      <c r="E13" s="10" t="n">
+        <v>0.000308</v>
+      </c>
+      <c r="F13" s="6" t="n">
+        <v>-5.2e-05</v>
+      </c>
+      <c r="G13" s="10" t="n">
+        <v>0.003345</v>
+      </c>
+      <c r="H13" s="6" t="n">
+        <v>-0.0001</v>
+      </c>
+      <c r="I13" s="6" t="n">
+        <v>-0.0009779999999999999</v>
+      </c>
+      <c r="J13" s="6" t="n">
+        <v>-0.0008129999999999999</v>
+      </c>
+      <c r="K13" s="10" t="n">
         <v>0.000299</v>
       </c>
-      <c r="D13" s="10" t="n">
-        <v>0.000308</v>
-      </c>
-      <c r="E13" s="5" t="n">
-        <v>-0.0008129999999999999</v>
-      </c>
-      <c r="F13" s="10" t="n">
+      <c r="L13" s="10" t="n">
         <v>0.000656</v>
       </c>
-      <c r="G13" s="5" t="n">
+      <c r="M13" s="6" t="n">
         <v>-0.000439</v>
       </c>
-      <c r="H13" s="5" t="n">
-        <v>-0.0001</v>
-      </c>
-      <c r="I13" s="5" t="n">
-        <v>-0.0009779999999999999</v>
-      </c>
-      <c r="J13" s="5" t="n">
-        <v>-0.000229</v>
-      </c>
-      <c r="K13" s="5" t="n">
-        <v>-5.2e-05</v>
-      </c>
-      <c r="L13" s="10" t="n">
+      <c r="N13" s="10" t="n">
         <v>4e-05</v>
       </c>
-      <c r="M13" s="10" t="n">
-        <v>0.000246</v>
-      </c>
-      <c r="N13" s="10" t="n">
-        <v>0.003345</v>
-      </c>
+      <c r="O13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -1591,20 +1607,20 @@
       <c r="B14" s="9" t="n">
         <v>0</v>
       </c>
-      <c r="C14" s="10" t="n">
-        <v>0.001038</v>
-      </c>
-      <c r="D14" s="5" t="n">
+      <c r="C14" s="6" t="n">
+        <v>-0.000492</v>
+      </c>
+      <c r="D14" s="10" t="n">
+        <v>0.001373</v>
+      </c>
+      <c r="E14" s="6" t="n">
         <v>-0.0006980000000000001</v>
       </c>
-      <c r="E14" s="10" t="n">
-        <v>0.002991</v>
-      </c>
-      <c r="F14" s="10" t="n">
-        <v>0.001442</v>
+      <c r="F14" s="6" t="n">
+        <v>-0.0018</v>
       </c>
       <c r="G14" s="10" t="n">
-        <v>0.001477</v>
+        <v>0.001232</v>
       </c>
       <c r="H14" s="10" t="n">
         <v>0.0009959999999999999</v>
@@ -1613,20 +1629,21 @@
         <v>0.000974</v>
       </c>
       <c r="J14" s="10" t="n">
-        <v>0.001373</v>
-      </c>
-      <c r="K14" s="5" t="n">
-        <v>-0.0018</v>
+        <v>0.002991</v>
+      </c>
+      <c r="K14" s="10" t="n">
+        <v>0.001038</v>
       </c>
       <c r="L14" s="10" t="n">
+        <v>0.001442</v>
+      </c>
+      <c r="M14" s="10" t="n">
+        <v>0.001477</v>
+      </c>
+      <c r="N14" s="10" t="n">
         <v>0.00098</v>
       </c>
-      <c r="M14" s="5" t="n">
-        <v>-0.000492</v>
-      </c>
-      <c r="N14" s="10" t="n">
-        <v>0.001232</v>
-      </c>
+      <c r="O14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1634,45 +1651,46 @@
           <t>2026-02-20</t>
         </is>
       </c>
-      <c r="B15" s="5" t="n">
+      <c r="B15" s="6" t="n">
         <v>-0.0005</v>
       </c>
-      <c r="C15" s="10" t="n">
-        <v>0.0004660000000000001</v>
-      </c>
-      <c r="D15" s="10" t="n">
+      <c r="C15" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="D15" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="E15" s="10" t="n">
         <v>0.000196</v>
       </c>
-      <c r="E15" s="5" t="n">
-        <v>-0.002062</v>
-      </c>
-      <c r="F15" s="10" t="n">
-        <v>0.000528</v>
-      </c>
-      <c r="G15" s="5" t="n">
-        <v>-4.5e-05</v>
-      </c>
-      <c r="H15" s="5" t="n">
+      <c r="F15" s="6" t="n">
+        <v>-0.002574</v>
+      </c>
+      <c r="G15" s="10" t="n">
+        <v>0.002919</v>
+      </c>
+      <c r="H15" s="6" t="n">
         <v>-0.000495</v>
       </c>
       <c r="I15" s="10" t="n">
         <v>0.00049</v>
       </c>
-      <c r="J15" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="K15" s="5" t="n">
-        <v>-0.002574</v>
+      <c r="J15" s="6" t="n">
+        <v>-0.002062</v>
+      </c>
+      <c r="K15" s="10" t="n">
+        <v>0.0004660000000000001</v>
       </c>
       <c r="L15" s="10" t="n">
+        <v>0.000528</v>
+      </c>
+      <c r="M15" s="6" t="n">
+        <v>-4.5e-05</v>
+      </c>
+      <c r="N15" s="10" t="n">
         <v>0.000445</v>
       </c>
-      <c r="M15" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="N15" s="10" t="n">
-        <v>0.002919</v>
-      </c>
+      <c r="O15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -1683,20 +1701,20 @@
       <c r="B16" s="9" t="n">
         <v>0</v>
       </c>
-      <c r="C16" s="5" t="n">
-        <v>-0.000185</v>
-      </c>
-      <c r="D16" s="5" t="n">
+      <c r="C16" s="10" t="n">
+        <v>0.0004929999999999999</v>
+      </c>
+      <c r="D16" s="10" t="n">
+        <v>0.000459</v>
+      </c>
+      <c r="E16" s="6" t="n">
         <v>-0.000935</v>
       </c>
-      <c r="E16" s="5" t="n">
-        <v>-0.000808</v>
-      </c>
       <c r="F16" s="10" t="n">
-        <v>0.000399</v>
+        <v>0.000914</v>
       </c>
       <c r="G16" s="10" t="n">
-        <v>0.0003500000000000001</v>
+        <v>0.001812</v>
       </c>
       <c r="H16" s="10" t="n">
         <v>0.0009970000000000001</v>
@@ -1704,21 +1722,22 @@
       <c r="I16" s="9" t="n">
         <v>0</v>
       </c>
-      <c r="J16" s="10" t="n">
-        <v>0.000459</v>
-      </c>
-      <c r="K16" s="10" t="n">
-        <v>0.000914</v>
+      <c r="J16" s="6" t="n">
+        <v>-0.000808</v>
+      </c>
+      <c r="K16" s="6" t="n">
+        <v>-0.000185</v>
       </c>
       <c r="L16" s="10" t="n">
+        <v>0.000399</v>
+      </c>
+      <c r="M16" s="10" t="n">
+        <v>0.0003500000000000001</v>
+      </c>
+      <c r="N16" s="10" t="n">
         <v>1e-05</v>
       </c>
-      <c r="M16" s="10" t="n">
-        <v>0.0004929999999999999</v>
-      </c>
-      <c r="N16" s="10" t="n">
-        <v>0.001812</v>
-      </c>
+      <c r="O16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -1729,42 +1748,43 @@
       <c r="B17" s="10" t="n">
         <v>0.0005</v>
       </c>
-      <c r="C17" s="5" t="n">
-        <v>-0.000273</v>
+      <c r="C17" s="6" t="n">
+        <v>-0.000492</v>
       </c>
       <c r="D17" s="10" t="n">
+        <v>0.000225</v>
+      </c>
+      <c r="E17" s="10" t="n">
         <v>0.000175</v>
       </c>
-      <c r="E17" s="5" t="n">
-        <v>-0.0005419999999999999</v>
-      </c>
-      <c r="F17" s="5" t="n">
-        <v>-0.000409</v>
+      <c r="F17" s="10" t="n">
+        <v>0.000915</v>
       </c>
       <c r="G17" s="10" t="n">
-        <v>0.000914</v>
-      </c>
-      <c r="H17" s="5" t="n">
+        <v>0.001661</v>
+      </c>
+      <c r="H17" s="6" t="n">
         <v>-0.001496</v>
       </c>
       <c r="I17" s="10" t="n">
         <v>0.0009750000000000001</v>
       </c>
-      <c r="J17" s="10" t="n">
-        <v>0.000225</v>
-      </c>
-      <c r="K17" s="10" t="n">
-        <v>0.000915</v>
-      </c>
-      <c r="L17" s="10" t="n">
+      <c r="J17" s="6" t="n">
+        <v>-0.0005419999999999999</v>
+      </c>
+      <c r="K17" s="6" t="n">
+        <v>-0.000273</v>
+      </c>
+      <c r="L17" s="6" t="n">
+        <v>-0.000409</v>
+      </c>
+      <c r="M17" s="10" t="n">
+        <v>0.000914</v>
+      </c>
+      <c r="N17" s="10" t="n">
         <v>0.000283</v>
       </c>
-      <c r="M17" s="5" t="n">
-        <v>-0.000492</v>
-      </c>
-      <c r="N17" s="10" t="n">
-        <v>0.001661</v>
-      </c>
+      <c r="O17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -1772,45 +1792,46 @@
           <t>2026-02-17</t>
         </is>
       </c>
-      <c r="B18" s="5" t="n">
+      <c r="B18" s="6" t="n">
         <v>-0.0005</v>
       </c>
-      <c r="C18" s="10" t="n">
-        <v>0.001083</v>
+      <c r="C18" s="6" t="n">
+        <v>-0.000487</v>
       </c>
       <c r="D18" s="10" t="n">
+        <v>0.0006900000000000001</v>
+      </c>
+      <c r="E18" s="10" t="n">
         <v>0.0009220000000000001</v>
       </c>
-      <c r="E18" s="10" t="n">
-        <v>0.001351</v>
-      </c>
-      <c r="F18" s="10" t="n">
-        <v>0.0011</v>
-      </c>
-      <c r="G18" s="10" t="n">
-        <v>0.000339</v>
+      <c r="F18" s="6" t="n">
+        <v>-3.1e-05</v>
+      </c>
+      <c r="G18" s="6" t="n">
+        <v>-0.001427</v>
       </c>
       <c r="H18" s="10" t="n">
         <v>0.001498</v>
       </c>
-      <c r="I18" s="5" t="n">
+      <c r="I18" s="6" t="n">
         <v>-0.0009750000000000001</v>
       </c>
       <c r="J18" s="10" t="n">
-        <v>0.0006900000000000001</v>
-      </c>
-      <c r="K18" s="5" t="n">
-        <v>-3.1e-05</v>
+        <v>0.001351</v>
+      </c>
+      <c r="K18" s="10" t="n">
+        <v>0.001083</v>
       </c>
       <c r="L18" s="10" t="n">
+        <v>0.0011</v>
+      </c>
+      <c r="M18" s="10" t="n">
+        <v>0.000339</v>
+      </c>
+      <c r="N18" s="10" t="n">
         <v>0.000779</v>
       </c>
-      <c r="M18" s="5" t="n">
-        <v>-0.000487</v>
-      </c>
-      <c r="N18" s="5" t="n">
-        <v>-0.001427</v>
-      </c>
+      <c r="O18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -1822,19 +1843,19 @@
         <v>0.0005</v>
       </c>
       <c r="C19" s="10" t="n">
-        <v>0.001579</v>
+        <v>0.001474</v>
       </c>
       <c r="D19" s="10" t="n">
+        <v>0.000916</v>
+      </c>
+      <c r="E19" s="10" t="n">
         <v>0.001245</v>
       </c>
-      <c r="E19" s="10" t="n">
-        <v>0.00217</v>
-      </c>
-      <c r="F19" s="10" t="n">
-        <v>0.001566</v>
+      <c r="F19" s="6" t="n">
+        <v>-0.000114</v>
       </c>
       <c r="G19" s="10" t="n">
-        <v>0.001051</v>
+        <v>0.004117</v>
       </c>
       <c r="H19" s="10" t="n">
         <v>0.002501</v>
@@ -1843,20 +1864,21 @@
         <v>0.001958</v>
       </c>
       <c r="J19" s="10" t="n">
-        <v>0.000916</v>
-      </c>
-      <c r="K19" s="5" t="n">
-        <v>-0.000114</v>
+        <v>0.00217</v>
+      </c>
+      <c r="K19" s="10" t="n">
+        <v>0.001579</v>
       </c>
       <c r="L19" s="10" t="n">
+        <v>0.001566</v>
+      </c>
+      <c r="M19" s="10" t="n">
+        <v>0.001051</v>
+      </c>
+      <c r="N19" s="10" t="n">
         <v>0.001012</v>
       </c>
-      <c r="M19" s="10" t="n">
-        <v>0.001474</v>
-      </c>
-      <c r="N19" s="10" t="n">
-        <v>0.004117</v>
-      </c>
+      <c r="O19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -1867,20 +1889,20 @@
       <c r="B20" s="10" t="n">
         <v>0.0009959999999999999</v>
       </c>
-      <c r="C20" s="10" t="n">
-        <v>0.002042</v>
+      <c r="C20" s="6" t="n">
+        <v>-0.001472</v>
       </c>
       <c r="D20" s="10" t="n">
+        <v>0.001609</v>
+      </c>
+      <c r="E20" s="10" t="n">
         <v>0.001499</v>
       </c>
-      <c r="E20" s="10" t="n">
-        <v>0.001896</v>
-      </c>
-      <c r="F20" s="10" t="n">
-        <v>0.002729</v>
-      </c>
-      <c r="G20" s="10" t="n">
-        <v>0.002834</v>
+      <c r="F20" s="6" t="n">
+        <v>-0.000644</v>
+      </c>
+      <c r="G20" s="6" t="n">
+        <v>-0.003159</v>
       </c>
       <c r="H20" s="10" t="n">
         <v>0.005032</v>
@@ -1889,20 +1911,21 @@
         <v>0.00245</v>
       </c>
       <c r="J20" s="10" t="n">
-        <v>0.001609</v>
-      </c>
-      <c r="K20" s="5" t="n">
-        <v>-0.000644</v>
+        <v>0.001896</v>
+      </c>
+      <c r="K20" s="10" t="n">
+        <v>0.002042</v>
       </c>
       <c r="L20" s="10" t="n">
+        <v>0.002729</v>
+      </c>
+      <c r="M20" s="10" t="n">
+        <v>0.002834</v>
+      </c>
+      <c r="N20" s="10" t="n">
         <v>0.002059</v>
       </c>
-      <c r="M20" s="5" t="n">
-        <v>-0.001472</v>
-      </c>
-      <c r="N20" s="5" t="n">
-        <v>-0.003159</v>
-      </c>
+      <c r="O20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -1914,41 +1937,42 @@
         <v>0</v>
       </c>
       <c r="C21" s="10" t="n">
-        <v>0.001026</v>
+        <v>0.001227</v>
       </c>
       <c r="D21" s="10" t="n">
+        <v>0.000692</v>
+      </c>
+      <c r="E21" s="10" t="n">
         <v>0.000575</v>
       </c>
-      <c r="E21" s="5" t="n">
-        <v>-0.000267</v>
-      </c>
-      <c r="F21" s="5" t="n">
-        <v>-0.00013</v>
-      </c>
-      <c r="G21" s="5" t="n">
-        <v>-0.000578</v>
-      </c>
-      <c r="H21" s="5" t="n">
+      <c r="F21" s="10" t="n">
+        <v>0.0008630000000000001</v>
+      </c>
+      <c r="G21" s="10" t="n">
+        <v>0.003183</v>
+      </c>
+      <c r="H21" s="6" t="n">
         <v>-0.001507</v>
       </c>
       <c r="I21" s="10" t="n">
         <v>0.000492</v>
       </c>
-      <c r="J21" s="10" t="n">
-        <v>0.000692</v>
+      <c r="J21" s="6" t="n">
+        <v>-0.000267</v>
       </c>
       <c r="K21" s="10" t="n">
-        <v>0.0008630000000000001</v>
-      </c>
-      <c r="L21" s="10" t="n">
+        <v>0.001026</v>
+      </c>
+      <c r="L21" s="6" t="n">
+        <v>-0.00013</v>
+      </c>
+      <c r="M21" s="6" t="n">
+        <v>-0.000578</v>
+      </c>
+      <c r="N21" s="10" t="n">
         <v>0.000365</v>
       </c>
-      <c r="M21" s="10" t="n">
-        <v>0.001227</v>
-      </c>
-      <c r="N21" s="10" t="n">
-        <v>0.003183</v>
-      </c>
+      <c r="O21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -1960,19 +1984,19 @@
         <v>0.001002</v>
       </c>
       <c r="C22" s="10" t="n">
-        <v>0.001347</v>
+        <v>0.000246</v>
       </c>
       <c r="D22" s="10" t="n">
+        <v>0.000919</v>
+      </c>
+      <c r="E22" s="10" t="n">
         <v>0.001327</v>
       </c>
-      <c r="E22" s="10" t="n">
-        <v>0.00054</v>
-      </c>
       <c r="F22" s="10" t="n">
-        <v>0.002638</v>
+        <v>0.001353</v>
       </c>
       <c r="G22" s="10" t="n">
-        <v>0.001055</v>
+        <v>0.002007</v>
       </c>
       <c r="H22" s="10" t="n">
         <v>0.003023</v>
@@ -1981,20 +2005,21 @@
         <v>0.000487</v>
       </c>
       <c r="J22" s="10" t="n">
-        <v>0.000919</v>
+        <v>0.00054</v>
       </c>
       <c r="K22" s="10" t="n">
-        <v>0.001353</v>
+        <v>0.001347</v>
       </c>
       <c r="L22" s="10" t="n">
+        <v>0.002638</v>
+      </c>
+      <c r="M22" s="10" t="n">
+        <v>0.001055</v>
+      </c>
+      <c r="N22" s="10" t="n">
         <v>0.001219</v>
       </c>
-      <c r="M22" s="10" t="n">
-        <v>0.000246</v>
-      </c>
-      <c r="N22" s="10" t="n">
-        <v>0.002007</v>
-      </c>
+      <c r="O22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -2006,41 +2031,42 @@
         <v>0</v>
       </c>
       <c r="C23" s="10" t="n">
-        <v>0.000683</v>
+        <v>0.001471</v>
       </c>
       <c r="D23" s="10" t="n">
+        <v>0.000462</v>
+      </c>
+      <c r="E23" s="10" t="n">
         <v>0.000239</v>
       </c>
-      <c r="E23" s="10" t="n">
-        <v>0.001632</v>
-      </c>
-      <c r="F23" s="10" t="n">
-        <v>0.000163</v>
+      <c r="F23" s="6" t="n">
+        <v>-0.004282</v>
       </c>
       <c r="G23" s="10" t="n">
-        <v>0.000113</v>
-      </c>
-      <c r="H23" s="5" t="n">
+        <v>0.001671</v>
+      </c>
+      <c r="H23" s="6" t="n">
         <v>-0.000505</v>
       </c>
       <c r="I23" s="10" t="n">
         <v>0.0004929999999999999</v>
       </c>
       <c r="J23" s="10" t="n">
-        <v>0.000462</v>
-      </c>
-      <c r="K23" s="5" t="n">
-        <v>-0.004282</v>
-      </c>
-      <c r="L23" s="5" t="n">
+        <v>0.001632</v>
+      </c>
+      <c r="K23" s="10" t="n">
+        <v>0.000683</v>
+      </c>
+      <c r="L23" s="10" t="n">
+        <v>0.000163</v>
+      </c>
+      <c r="M23" s="10" t="n">
+        <v>0.000113</v>
+      </c>
+      <c r="N23" s="6" t="n">
         <v>-0.000163</v>
       </c>
-      <c r="M23" s="10" t="n">
-        <v>0.001471</v>
-      </c>
-      <c r="N23" s="10" t="n">
-        <v>0.001671</v>
-      </c>
+      <c r="O23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -2051,20 +2077,20 @@
       <c r="B24" s="10" t="n">
         <v>0.000998</v>
       </c>
-      <c r="C24" s="10" t="n">
-        <v>0.000364</v>
+      <c r="C24" s="9" t="n">
+        <v>0</v>
       </c>
       <c r="D24" s="10" t="n">
+        <v>0.000458</v>
+      </c>
+      <c r="E24" s="10" t="n">
         <v>0.000513</v>
       </c>
-      <c r="E24" s="10" t="n">
-        <v>0.001635</v>
-      </c>
-      <c r="F24" s="10" t="n">
-        <v>0.000511</v>
+      <c r="F24" s="6" t="n">
+        <v>-0.002038</v>
       </c>
       <c r="G24" s="10" t="n">
-        <v>0.000499</v>
+        <v>0.005980999999999999</v>
       </c>
       <c r="H24" s="10" t="n">
         <v>0.000505</v>
@@ -2073,20 +2099,21 @@
         <v>0.0009810000000000001</v>
       </c>
       <c r="J24" s="10" t="n">
-        <v>0.000458</v>
-      </c>
-      <c r="K24" s="5" t="n">
-        <v>-0.002038</v>
+        <v>0.001635</v>
+      </c>
+      <c r="K24" s="10" t="n">
+        <v>0.000364</v>
       </c>
       <c r="L24" s="10" t="n">
+        <v>0.000511</v>
+      </c>
+      <c r="M24" s="10" t="n">
+        <v>0.000499</v>
+      </c>
+      <c r="N24" s="10" t="n">
         <v>0.000163</v>
       </c>
-      <c r="M24" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="N24" s="10" t="n">
-        <v>0.005980999999999999</v>
-      </c>
+      <c r="O24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -2094,23 +2121,23 @@
           <t>2026-02-05</t>
         </is>
       </c>
-      <c r="B25" s="5" t="n">
+      <c r="B25" s="6" t="n">
         <v>-0.001497</v>
       </c>
-      <c r="C25" s="10" t="n">
-        <v>0.0009229999999999999</v>
+      <c r="C25" s="9" t="n">
+        <v>0</v>
       </c>
       <c r="D25" s="10" t="n">
+        <v>0.002772</v>
+      </c>
+      <c r="E25" s="10" t="n">
         <v>0.000316</v>
       </c>
-      <c r="E25" s="10" t="n">
-        <v>0.000273</v>
-      </c>
-      <c r="F25" s="10" t="n">
-        <v>0.00197</v>
-      </c>
-      <c r="G25" s="10" t="n">
-        <v>0.0006469999999999999</v>
+      <c r="F25" s="6" t="n">
+        <v>-0.000879</v>
+      </c>
+      <c r="G25" s="6" t="n">
+        <v>-0.008935999999999999</v>
       </c>
       <c r="H25" s="10" t="n">
         <v>0.004555</v>
@@ -2119,20 +2146,21 @@
         <v>0.0004929999999999999</v>
       </c>
       <c r="J25" s="10" t="n">
-        <v>0.002772</v>
-      </c>
-      <c r="K25" s="5" t="n">
-        <v>-0.000879</v>
+        <v>0.000273</v>
+      </c>
+      <c r="K25" s="10" t="n">
+        <v>0.0009229999999999999</v>
       </c>
       <c r="L25" s="10" t="n">
+        <v>0.00197</v>
+      </c>
+      <c r="M25" s="10" t="n">
+        <v>0.0006469999999999999</v>
+      </c>
+      <c r="N25" s="10" t="n">
         <v>0.001058</v>
       </c>
-      <c r="M25" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="N25" s="5" t="n">
-        <v>-0.008935999999999999</v>
-      </c>
+      <c r="O25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -2143,42 +2171,43 @@
       <c r="B26" s="10" t="n">
         <v>0.001002</v>
       </c>
-      <c r="C26" s="5" t="n">
-        <v>-0.00047</v>
-      </c>
-      <c r="D26" s="10" t="n">
+      <c r="C26" s="10" t="n">
+        <v>0.000494</v>
+      </c>
+      <c r="D26" s="6" t="n">
+        <v>-0.001384</v>
+      </c>
+      <c r="E26" s="10" t="n">
         <v>0.000183</v>
       </c>
-      <c r="E26" s="5" t="n">
-        <v>-0.000273</v>
-      </c>
       <c r="F26" s="10" t="n">
-        <v>4.400000000000001e-05</v>
-      </c>
-      <c r="G26" s="10" t="n">
-        <v>0.000432</v>
-      </c>
-      <c r="H26" s="5" t="n">
+        <v>0.0006619999999999999</v>
+      </c>
+      <c r="G26" s="6" t="n">
+        <v>-0.001124</v>
+      </c>
+      <c r="H26" s="6" t="n">
         <v>-0.001009</v>
       </c>
       <c r="I26" s="10" t="n">
         <v>0.000494</v>
       </c>
-      <c r="J26" s="5" t="n">
-        <v>-0.001384</v>
-      </c>
-      <c r="K26" s="10" t="n">
-        <v>0.0006619999999999999</v>
+      <c r="J26" s="6" t="n">
+        <v>-0.000273</v>
+      </c>
+      <c r="K26" s="6" t="n">
+        <v>-0.00047</v>
       </c>
       <c r="L26" s="10" t="n">
+        <v>4.400000000000001e-05</v>
+      </c>
+      <c r="M26" s="10" t="n">
+        <v>0.000432</v>
+      </c>
+      <c r="N26" s="10" t="n">
         <v>0.000122</v>
       </c>
-      <c r="M26" s="10" t="n">
-        <v>0.000494</v>
-      </c>
-      <c r="N26" s="5" t="n">
-        <v>-0.001124</v>
-      </c>
+      <c r="O26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -2186,45 +2215,46 @@
           <t>2026-02-03</t>
         </is>
       </c>
-      <c r="B27" s="5" t="n">
+      <c r="B27" s="6" t="n">
         <v>-0.000501</v>
       </c>
-      <c r="C27" s="10" t="n">
+      <c r="C27" s="6" t="n">
+        <v>-0.000494</v>
+      </c>
+      <c r="D27" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="E27" s="6" t="n">
+        <v>-9.1e-05</v>
+      </c>
+      <c r="F27" s="10" t="n">
+        <v>0.0005899999999999999</v>
+      </c>
+      <c r="G27" s="10" t="n">
+        <v>0.00392</v>
+      </c>
+      <c r="H27" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="I27" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="J27" s="10" t="n">
+        <v>0.0008210000000000001</v>
+      </c>
+      <c r="K27" s="10" t="n">
         <v>0.000257</v>
       </c>
-      <c r="D27" s="5" t="n">
-        <v>-9.1e-05</v>
-      </c>
-      <c r="E27" s="10" t="n">
-        <v>0.0008210000000000001</v>
-      </c>
-      <c r="F27" s="5" t="n">
+      <c r="L27" s="6" t="n">
         <v>-1.1e-05</v>
       </c>
-      <c r="G27" s="5" t="n">
+      <c r="M27" s="6" t="n">
         <v>-0.000204</v>
       </c>
-      <c r="H27" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="I27" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="J27" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="K27" s="10" t="n">
-        <v>0.0005899999999999999</v>
-      </c>
-      <c r="L27" s="5" t="n">
+      <c r="N27" s="6" t="n">
         <v>-0.000122</v>
       </c>
-      <c r="M27" s="5" t="n">
-        <v>-0.000494</v>
-      </c>
-      <c r="N27" s="10" t="n">
-        <v>0.00392</v>
-      </c>
+      <c r="O27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -2235,42 +2265,43 @@
       <c r="B28" s="10" t="n">
         <v>0.000501</v>
       </c>
-      <c r="C28" s="10" t="n">
+      <c r="C28" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="D28" s="6" t="n">
+        <v>-0.000463</v>
+      </c>
+      <c r="E28" s="6" t="n">
+        <v>-6.3e-05</v>
+      </c>
+      <c r="F28" s="10" t="n">
+        <v>8.3e-05</v>
+      </c>
+      <c r="G28" s="10" t="n">
+        <v>7e-06</v>
+      </c>
+      <c r="H28" s="6" t="n">
+        <v>-0.001014</v>
+      </c>
+      <c r="I28" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="J28" s="6" t="n">
+        <v>-0.001361</v>
+      </c>
+      <c r="K28" s="10" t="n">
         <v>0.001244</v>
       </c>
-      <c r="D28" s="5" t="n">
-        <v>-6.3e-05</v>
-      </c>
-      <c r="E28" s="5" t="n">
-        <v>-0.001361</v>
-      </c>
-      <c r="F28" s="5" t="n">
+      <c r="L28" s="6" t="n">
         <v>-0.0009239999999999999</v>
       </c>
-      <c r="G28" s="10" t="n">
+      <c r="M28" s="10" t="n">
         <v>0.0005909999999999999</v>
       </c>
-      <c r="H28" s="5" t="n">
-        <v>-0.001014</v>
-      </c>
-      <c r="I28" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="J28" s="5" t="n">
-        <v>-0.000463</v>
-      </c>
-      <c r="K28" s="10" t="n">
-        <v>8.3e-05</v>
-      </c>
-      <c r="L28" s="10" t="n">
+      <c r="N28" s="10" t="n">
         <v>0.000376</v>
       </c>
-      <c r="M28" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="N28" s="10" t="n">
-        <v>7e-06</v>
-      </c>
+      <c r="O28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -2281,42 +2312,43 @@
       <c r="B29" s="9" t="n">
         <v>0</v>
       </c>
-      <c r="C29" s="5" t="n">
+      <c r="C29" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="D29" s="10" t="n">
+        <v>0.0009260000000000001</v>
+      </c>
+      <c r="E29" s="6" t="n">
+        <v>-0.000239</v>
+      </c>
+      <c r="F29" s="6" t="n">
+        <v>-0.001354</v>
+      </c>
+      <c r="G29" s="6" t="n">
+        <v>-0.011534</v>
+      </c>
+      <c r="H29" s="6" t="n">
+        <v>-0.000501</v>
+      </c>
+      <c r="I29" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="J29" s="6" t="n">
+        <v>-0.002176</v>
+      </c>
+      <c r="K29" s="6" t="n">
         <v>-0.00079</v>
       </c>
-      <c r="D29" s="5" t="n">
-        <v>-0.000239</v>
-      </c>
-      <c r="E29" s="5" t="n">
-        <v>-0.002176</v>
-      </c>
-      <c r="F29" s="5" t="n">
+      <c r="L29" s="6" t="n">
         <v>-0.000619</v>
       </c>
-      <c r="G29" s="5" t="n">
+      <c r="M29" s="6" t="n">
         <v>-0.000398</v>
       </c>
-      <c r="H29" s="5" t="n">
-        <v>-0.000501</v>
-      </c>
-      <c r="I29" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="J29" s="10" t="n">
-        <v>0.0009260000000000001</v>
-      </c>
-      <c r="K29" s="5" t="n">
-        <v>-0.001354</v>
-      </c>
-      <c r="L29" s="10" t="n">
+      <c r="N29" s="10" t="n">
         <v>0.000428</v>
       </c>
-      <c r="M29" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="N29" s="5" t="n">
-        <v>-0.011534</v>
-      </c>
+      <c r="O29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -2327,20 +2359,20 @@
       <c r="B30" s="10" t="n">
         <v>0.000998</v>
       </c>
-      <c r="C30" s="5" t="n">
-        <v>-0.000337</v>
+      <c r="C30" s="10" t="n">
+        <v>0.0009829999999999999</v>
       </c>
       <c r="D30" s="10" t="n">
+        <v>0.0009220000000000001</v>
+      </c>
+      <c r="E30" s="10" t="n">
         <v>0.000309</v>
       </c>
-      <c r="E30" s="10" t="n">
-        <v>0.001633</v>
-      </c>
-      <c r="F30" s="10" t="n">
-        <v>0.000555</v>
-      </c>
-      <c r="G30" s="5" t="n">
-        <v>-0.000136</v>
+      <c r="F30" s="6" t="n">
+        <v>-0.000548</v>
+      </c>
+      <c r="G30" s="6" t="n">
+        <v>-0.002343</v>
       </c>
       <c r="H30" s="10" t="n">
         <v>0.0005020000000000001</v>
@@ -2349,20 +2381,21 @@
         <v>0.0009829999999999999</v>
       </c>
       <c r="J30" s="10" t="n">
-        <v>0.0009220000000000001</v>
-      </c>
-      <c r="K30" s="5" t="n">
-        <v>-0.000548</v>
-      </c>
-      <c r="L30" s="5" t="n">
+        <v>0.001633</v>
+      </c>
+      <c r="K30" s="6" t="n">
+        <v>-0.000337</v>
+      </c>
+      <c r="L30" s="10" t="n">
+        <v>0.000555</v>
+      </c>
+      <c r="M30" s="6" t="n">
+        <v>-0.000136</v>
+      </c>
+      <c r="N30" s="6" t="n">
         <v>-0.000204</v>
       </c>
-      <c r="M30" s="10" t="n">
-        <v>0.0009829999999999999</v>
-      </c>
-      <c r="N30" s="5" t="n">
-        <v>-0.002343</v>
-      </c>
+      <c r="O30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -2373,42 +2406,43 @@
       <c r="B31" s="9" t="n">
         <v>0</v>
       </c>
-      <c r="C31" s="5" t="n">
-        <v>-0.000497</v>
-      </c>
-      <c r="D31" s="5" t="n">
+      <c r="C31" s="10" t="n">
+        <v>0.000494</v>
+      </c>
+      <c r="D31" s="10" t="n">
+        <v>0.0004639999999999999</v>
+      </c>
+      <c r="E31" s="6" t="n">
         <v>-4.9e-05</v>
       </c>
-      <c r="E31" s="10" t="n">
-        <v>0.002184</v>
-      </c>
-      <c r="F31" s="5" t="n">
-        <v>-2.2e-05</v>
-      </c>
-      <c r="G31" s="5" t="n">
-        <v>-0.00101</v>
-      </c>
-      <c r="H31" s="5" t="n">
+      <c r="F31" s="10" t="n">
+        <v>0.000837</v>
+      </c>
+      <c r="G31" s="10" t="n">
+        <v>0.002943</v>
+      </c>
+      <c r="H31" s="6" t="n">
         <v>-0.001513</v>
       </c>
       <c r="I31" s="10" t="n">
         <v>0.000494</v>
       </c>
       <c r="J31" s="10" t="n">
-        <v>0.0004639999999999999</v>
-      </c>
-      <c r="K31" s="10" t="n">
-        <v>0.000837</v>
-      </c>
-      <c r="L31" s="5" t="n">
+        <v>0.002184</v>
+      </c>
+      <c r="K31" s="6" t="n">
+        <v>-0.000497</v>
+      </c>
+      <c r="L31" s="6" t="n">
+        <v>-2.2e-05</v>
+      </c>
+      <c r="M31" s="6" t="n">
+        <v>-0.00101</v>
+      </c>
+      <c r="N31" s="6" t="n">
         <v>-0.000285</v>
       </c>
-      <c r="M31" s="10" t="n">
-        <v>0.000494</v>
-      </c>
-      <c r="N31" s="10" t="n">
-        <v>0.002943</v>
-      </c>
+      <c r="O31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -2419,42 +2453,43 @@
       <c r="B32" s="10" t="n">
         <v>0.000452</v>
       </c>
-      <c r="C32" s="5" t="n">
+      <c r="C32" s="6" t="n">
+        <v>-0.00123</v>
+      </c>
+      <c r="D32" s="10" t="n">
+        <v>0.000232</v>
+      </c>
+      <c r="E32" s="6" t="n">
+        <v>-0.00073</v>
+      </c>
+      <c r="F32" s="6" t="n">
+        <v>-0.000992</v>
+      </c>
+      <c r="G32" s="10" t="n">
+        <v>0.000153</v>
+      </c>
+      <c r="H32" s="6" t="n">
+        <v>-0.002111</v>
+      </c>
+      <c r="I32" s="6" t="n">
+        <v>-0.001968</v>
+      </c>
+      <c r="J32" s="6" t="n">
+        <v>-0.002179</v>
+      </c>
+      <c r="K32" s="6" t="n">
         <v>-0.001072</v>
       </c>
-      <c r="D32" s="5" t="n">
-        <v>-0.00073</v>
-      </c>
-      <c r="E32" s="5" t="n">
-        <v>-0.002179</v>
-      </c>
-      <c r="F32" s="5" t="n">
+      <c r="L32" s="6" t="n">
         <v>-0.000739</v>
       </c>
-      <c r="G32" s="5" t="n">
+      <c r="M32" s="6" t="n">
         <v>-0.0009180000000000001</v>
       </c>
-      <c r="H32" s="5" t="n">
-        <v>-0.002111</v>
-      </c>
-      <c r="I32" s="5" t="n">
-        <v>-0.001968</v>
-      </c>
-      <c r="J32" s="10" t="n">
-        <v>0.000232</v>
-      </c>
-      <c r="K32" s="5" t="n">
-        <v>-0.000992</v>
-      </c>
-      <c r="L32" s="5" t="n">
+      <c r="N32" s="6" t="n">
         <v>-0.00126</v>
       </c>
-      <c r="M32" s="5" t="n">
-        <v>-0.00123</v>
-      </c>
-      <c r="N32" s="10" t="n">
-        <v>0.000153</v>
-      </c>
+      <c r="O32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -2466,19 +2501,19 @@
         <v>0.000497</v>
       </c>
       <c r="C33" s="10" t="n">
-        <v>0.001696</v>
-      </c>
-      <c r="D33" s="10" t="n">
+        <v>0.0009790000000000001</v>
+      </c>
+      <c r="D33" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="E33" s="10" t="n">
         <v>0.00197</v>
       </c>
-      <c r="E33" s="10" t="n">
-        <v>0.001088</v>
-      </c>
       <c r="F33" s="10" t="n">
-        <v>0.001949</v>
+        <v>0.000207</v>
       </c>
       <c r="G33" s="10" t="n">
-        <v>0.001067</v>
+        <v>0.004125</v>
       </c>
       <c r="H33" s="10" t="n">
         <v>0.001001</v>
@@ -2486,21 +2521,22 @@
       <c r="I33" s="10" t="n">
         <v>0.002949</v>
       </c>
-      <c r="J33" s="9" t="n">
-        <v>0</v>
+      <c r="J33" s="10" t="n">
+        <v>0.001088</v>
       </c>
       <c r="K33" s="10" t="n">
-        <v>0.000207</v>
+        <v>0.001696</v>
       </c>
       <c r="L33" s="10" t="n">
+        <v>0.001949</v>
+      </c>
+      <c r="M33" s="10" t="n">
+        <v>0.001067</v>
+      </c>
+      <c r="N33" s="10" t="n">
         <v>0.001822</v>
       </c>
-      <c r="M33" s="10" t="n">
-        <v>0.0009790000000000001</v>
-      </c>
-      <c r="N33" s="10" t="n">
-        <v>0.004125</v>
-      </c>
+      <c r="O33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -2511,42 +2547,43 @@
       <c r="B34" s="10" t="n">
         <v>0.0005020000000000001</v>
       </c>
-      <c r="C34" s="5" t="n">
-        <v>-0.000719</v>
-      </c>
-      <c r="D34" s="5" t="n">
+      <c r="C34" s="10" t="n">
+        <v>0.001961</v>
+      </c>
+      <c r="D34" s="10" t="n">
+        <v>0.000459</v>
+      </c>
+      <c r="E34" s="6" t="n">
         <v>-0.00038</v>
       </c>
-      <c r="E34" s="10" t="n">
-        <v>0.001912</v>
-      </c>
-      <c r="F34" s="10" t="n">
-        <v>0.000414</v>
-      </c>
-      <c r="G34" s="5" t="n">
-        <v>-0.000556</v>
+      <c r="F34" s="6" t="n">
+        <v>-0.000341</v>
+      </c>
+      <c r="G34" s="10" t="n">
+        <v>0.0007149999999999999</v>
       </c>
       <c r="H34" s="10" t="n">
         <v>0.0005059999999999999</v>
       </c>
-      <c r="I34" s="5" t="n">
+      <c r="I34" s="6" t="n">
         <v>-0.000495</v>
       </c>
       <c r="J34" s="10" t="n">
-        <v>0.000459</v>
-      </c>
-      <c r="K34" s="5" t="n">
-        <v>-0.000341</v>
-      </c>
-      <c r="L34" s="5" t="n">
+        <v>0.001912</v>
+      </c>
+      <c r="K34" s="6" t="n">
+        <v>-0.000719</v>
+      </c>
+      <c r="L34" s="10" t="n">
+        <v>0.000414</v>
+      </c>
+      <c r="M34" s="6" t="n">
+        <v>-0.000556</v>
+      </c>
+      <c r="N34" s="6" t="n">
         <v>-0.000326</v>
       </c>
-      <c r="M34" s="10" t="n">
-        <v>0.001961</v>
-      </c>
-      <c r="N34" s="10" t="n">
-        <v>0.0007149999999999999</v>
-      </c>
+      <c r="O34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -2558,19 +2595,19 @@
         <v>0</v>
       </c>
       <c r="C35" s="10" t="n">
-        <v>0.001493</v>
+        <v>0.000982</v>
       </c>
       <c r="D35" s="10" t="n">
+        <v>0.002307</v>
+      </c>
+      <c r="E35" s="10" t="n">
         <v>0.001437</v>
       </c>
-      <c r="E35" s="10" t="n">
-        <v>0.002521</v>
-      </c>
       <c r="F35" s="10" t="n">
-        <v>0.001167</v>
+        <v>0.001137</v>
       </c>
       <c r="G35" s="10" t="n">
-        <v>0.00067</v>
+        <v>0.005277</v>
       </c>
       <c r="H35" s="10" t="n">
         <v>0.002012</v>
@@ -2579,20 +2616,21 @@
         <v>0.001476</v>
       </c>
       <c r="J35" s="10" t="n">
-        <v>0.002307</v>
+        <v>0.002521</v>
       </c>
       <c r="K35" s="10" t="n">
-        <v>0.001137</v>
+        <v>0.001493</v>
       </c>
       <c r="L35" s="10" t="n">
+        <v>0.001167</v>
+      </c>
+      <c r="M35" s="10" t="n">
+        <v>0.00067</v>
+      </c>
+      <c r="N35" s="10" t="n">
         <v>0.000896</v>
       </c>
-      <c r="M35" s="10" t="n">
-        <v>0.000982</v>
-      </c>
-      <c r="N35" s="10" t="n">
-        <v>0.005277</v>
-      </c>
+      <c r="O35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -2603,20 +2641,20 @@
       <c r="B36" s="10" t="n">
         <v>0.000498</v>
       </c>
-      <c r="C36" s="10" t="n">
-        <v>0.001067</v>
-      </c>
-      <c r="D36" s="10" t="n">
+      <c r="C36" s="6" t="n">
+        <v>-0.000491</v>
+      </c>
+      <c r="D36" s="6" t="n">
+        <v>-0.00046</v>
+      </c>
+      <c r="E36" s="10" t="n">
         <v>0.00067</v>
       </c>
-      <c r="E36" s="5" t="n">
-        <v>-0.003813</v>
-      </c>
       <c r="F36" s="10" t="n">
-        <v>0.002229</v>
+        <v>0.000569</v>
       </c>
       <c r="G36" s="10" t="n">
-        <v>0.00166</v>
+        <v>0.003095</v>
       </c>
       <c r="H36" s="10" t="n">
         <v>0.006077</v>
@@ -2624,21 +2662,22 @@
       <c r="I36" s="10" t="n">
         <v>0.001478</v>
       </c>
-      <c r="J36" s="5" t="n">
-        <v>-0.00046</v>
+      <c r="J36" s="6" t="n">
+        <v>-0.003813</v>
       </c>
       <c r="K36" s="10" t="n">
-        <v>0.000569</v>
+        <v>0.001067</v>
       </c>
       <c r="L36" s="10" t="n">
+        <v>0.002229</v>
+      </c>
+      <c r="M36" s="10" t="n">
+        <v>0.00166</v>
+      </c>
+      <c r="N36" s="10" t="n">
         <v>0.001336</v>
       </c>
-      <c r="M36" s="5" t="n">
-        <v>-0.000491</v>
-      </c>
-      <c r="N36" s="10" t="n">
-        <v>0.003095</v>
-      </c>
+      <c r="O36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -2646,43 +2685,44 @@
           <t>2026-01-20</t>
         </is>
       </c>
-      <c r="B37" s="5" t="n">
+      <c r="B37" s="6" t="n">
         <v>-0.001496</v>
       </c>
-      <c r="C37" s="5" t="n">
+      <c r="C37" t="inlineStr"/>
+      <c r="D37" s="10" t="n">
+        <v>0.00046</v>
+      </c>
+      <c r="E37" s="6" t="n">
+        <v>-0.001632</v>
+      </c>
+      <c r="F37" s="6" t="n">
+        <v>-0.001745</v>
+      </c>
+      <c r="G37" s="10" t="n">
+        <v>0.000438</v>
+      </c>
+      <c r="H37" s="6" t="n">
+        <v>-0.012007</v>
+      </c>
+      <c r="I37" s="6" t="n">
+        <v>-0.001965</v>
+      </c>
+      <c r="J37" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="K37" s="6" t="n">
         <v>-0.002555</v>
       </c>
-      <c r="D37" s="5" t="n">
-        <v>-0.001632</v>
-      </c>
-      <c r="E37" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="F37" s="5" t="n">
+      <c r="L37" s="6" t="n">
         <v>-0.003853</v>
       </c>
-      <c r="G37" s="5" t="n">
+      <c r="M37" s="6" t="n">
         <v>-0.002642</v>
       </c>
-      <c r="H37" s="5" t="n">
-        <v>-0.012007</v>
-      </c>
-      <c r="I37" s="5" t="n">
-        <v>-0.001965</v>
-      </c>
-      <c r="J37" s="10" t="n">
-        <v>0.00046</v>
-      </c>
-      <c r="K37" s="5" t="n">
-        <v>-0.001745</v>
-      </c>
-      <c r="L37" s="5" t="n">
+      <c r="N37" s="6" t="n">
         <v>-0.002249</v>
       </c>
-      <c r="M37" t="inlineStr"/>
-      <c r="N37" s="10" t="n">
-        <v>0.000438</v>
-      </c>
+      <c r="O37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -2693,40 +2733,41 @@
       <c r="B38" s="9" t="n">
         <v>0</v>
       </c>
-      <c r="C38" s="5" t="n">
-        <v>-0.000355</v>
-      </c>
-      <c r="D38" s="5" t="n">
+      <c r="C38" t="inlineStr"/>
+      <c r="D38" s="6" t="n">
+        <v>-0.001379</v>
+      </c>
+      <c r="E38" s="6" t="n">
         <v>-0.000295</v>
       </c>
-      <c r="E38" s="5" t="n">
-        <v>-0.002712</v>
-      </c>
-      <c r="F38" s="5" t="n">
-        <v>-0.001066</v>
-      </c>
-      <c r="G38" s="5" t="n">
-        <v>-0.000215</v>
+      <c r="F38" s="10" t="n">
+        <v>0.000527</v>
+      </c>
+      <c r="G38" s="10" t="n">
+        <v>0.000906</v>
       </c>
       <c r="H38" s="10" t="n">
         <v>0.005536</v>
       </c>
-      <c r="I38" s="5" t="n">
+      <c r="I38" s="6" t="n">
         <v>-0.0009840000000000001</v>
       </c>
-      <c r="J38" s="5" t="n">
-        <v>-0.001379</v>
-      </c>
-      <c r="K38" s="10" t="n">
-        <v>0.000527</v>
-      </c>
-      <c r="L38" s="5" t="n">
+      <c r="J38" s="6" t="n">
+        <v>-0.002712</v>
+      </c>
+      <c r="K38" s="6" t="n">
+        <v>-0.000355</v>
+      </c>
+      <c r="L38" s="6" t="n">
+        <v>-0.001066</v>
+      </c>
+      <c r="M38" s="6" t="n">
+        <v>-0.000215</v>
+      </c>
+      <c r="N38" s="6" t="n">
         <v>-0.000478</v>
       </c>
-      <c r="M38" t="inlineStr"/>
-      <c r="N38" s="10" t="n">
-        <v>0.000906</v>
-      </c>
+      <c r="O38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -2737,40 +2778,41 @@
       <c r="B39" s="9" t="n">
         <v>0</v>
       </c>
-      <c r="C39" s="5" t="n">
+      <c r="C39" t="inlineStr"/>
+      <c r="D39" s="6" t="n">
+        <v>-0.0004639999999999999</v>
+      </c>
+      <c r="E39" s="6" t="n">
+        <v>-0.000787</v>
+      </c>
+      <c r="F39" s="10" t="n">
+        <v>0.000724</v>
+      </c>
+      <c r="G39" s="6" t="n">
+        <v>-0.001343</v>
+      </c>
+      <c r="H39" s="6" t="n">
+        <v>-0.002511</v>
+      </c>
+      <c r="I39" s="6" t="n">
+        <v>-0.0009779999999999999</v>
+      </c>
+      <c r="J39" s="10" t="n">
+        <v>0.002176</v>
+      </c>
+      <c r="K39" s="6" t="n">
         <v>-0.0006469999999999999</v>
       </c>
-      <c r="D39" s="5" t="n">
-        <v>-0.000787</v>
-      </c>
-      <c r="E39" s="10" t="n">
-        <v>0.002176</v>
-      </c>
-      <c r="F39" s="5" t="n">
+      <c r="L39" s="6" t="n">
         <v>-0.001542</v>
       </c>
-      <c r="G39" s="5" t="n">
+      <c r="M39" s="6" t="n">
         <v>-0.001268</v>
       </c>
-      <c r="H39" s="5" t="n">
-        <v>-0.002511</v>
-      </c>
-      <c r="I39" s="5" t="n">
-        <v>-0.0009779999999999999</v>
-      </c>
-      <c r="J39" s="5" t="n">
-        <v>-0.0004639999999999999</v>
-      </c>
-      <c r="K39" s="10" t="n">
-        <v>0.000724</v>
-      </c>
-      <c r="L39" s="5" t="n">
+      <c r="N39" s="6" t="n">
         <v>-0.000661</v>
       </c>
-      <c r="M39" t="inlineStr"/>
-      <c r="N39" s="5" t="n">
-        <v>-0.001343</v>
-      </c>
+      <c r="O39" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -2781,40 +2823,41 @@
       <c r="B40" s="10" t="n">
         <v>0.000497</v>
       </c>
-      <c r="C40" s="10" t="n">
-        <v>0.00023</v>
-      </c>
+      <c r="C40" t="inlineStr"/>
       <c r="D40" s="10" t="n">
+        <v>0.000925</v>
+      </c>
+      <c r="E40" s="10" t="n">
         <v>0.000746</v>
       </c>
-      <c r="E40" s="5" t="n">
-        <v>-0.001632</v>
-      </c>
-      <c r="F40" s="5" t="n">
-        <v>-0.000293</v>
+      <c r="F40" s="10" t="n">
+        <v>0.000724</v>
       </c>
       <c r="G40" s="10" t="n">
-        <v>0.00026</v>
-      </c>
-      <c r="H40" s="5" t="n">
+        <v>0.000467</v>
+      </c>
+      <c r="H40" s="6" t="n">
         <v>-0.001503</v>
       </c>
       <c r="I40" s="10" t="n">
         <v>0.002457</v>
       </c>
-      <c r="J40" s="10" t="n">
-        <v>0.000925</v>
+      <c r="J40" s="6" t="n">
+        <v>-0.001632</v>
       </c>
       <c r="K40" s="10" t="n">
-        <v>0.000724</v>
-      </c>
-      <c r="L40" s="10" t="n">
+        <v>0.00023</v>
+      </c>
+      <c r="L40" s="6" t="n">
+        <v>-0.000293</v>
+      </c>
+      <c r="M40" s="10" t="n">
+        <v>0.00026</v>
+      </c>
+      <c r="N40" s="10" t="n">
         <v>0.00057</v>
       </c>
-      <c r="M40" t="inlineStr"/>
-      <c r="N40" s="10" t="n">
-        <v>0.000467</v>
-      </c>
+      <c r="O40" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -2825,20 +2868,18 @@
       <c r="B41" s="10" t="n">
         <v>0.0005020000000000001</v>
       </c>
-      <c r="C41" s="10" t="n">
-        <v>0.0007630000000000001</v>
-      </c>
+      <c r="C41" t="inlineStr"/>
       <c r="D41" s="10" t="n">
+        <v>0.00231</v>
+      </c>
+      <c r="E41" s="10" t="n">
         <v>0.001465</v>
       </c>
-      <c r="E41" s="10" t="n">
-        <v>0.000546</v>
-      </c>
       <c r="F41" s="10" t="n">
-        <v>0.001337</v>
+        <v>0.000311</v>
       </c>
       <c r="G41" s="10" t="n">
-        <v>0.0016</v>
+        <v>0.001147</v>
       </c>
       <c r="H41" s="10" t="n">
         <v>0.002513</v>
@@ -2847,18 +2888,21 @@
         <v>0.001975</v>
       </c>
       <c r="J41" s="10" t="n">
-        <v>0.00231</v>
+        <v>0.000546</v>
       </c>
       <c r="K41" s="10" t="n">
-        <v>0.000311</v>
+        <v>0.0007630000000000001</v>
       </c>
       <c r="L41" s="10" t="n">
+        <v>0.001337</v>
+      </c>
+      <c r="M41" s="10" t="n">
+        <v>0.0016</v>
+      </c>
+      <c r="N41" s="10" t="n">
         <v>0.001375</v>
       </c>
-      <c r="M41" t="inlineStr"/>
-      <c r="N41" s="10" t="n">
-        <v>0.001147</v>
-      </c>
+      <c r="O41" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -2869,40 +2913,41 @@
       <c r="B42" s="9" t="n">
         <v>0</v>
       </c>
-      <c r="C42" s="10" t="n">
-        <v>0.000319</v>
-      </c>
-      <c r="D42" s="10" t="n">
+      <c r="C42" t="inlineStr"/>
+      <c r="D42" s="6" t="n">
+        <v>-0.000461</v>
+      </c>
+      <c r="E42" s="10" t="n">
         <v>5.6e-05</v>
       </c>
-      <c r="E42" s="10" t="n">
-        <v>0.002997</v>
-      </c>
-      <c r="F42" s="5" t="n">
-        <v>-0.000684</v>
+      <c r="F42" s="10" t="n">
+        <v>0.000964</v>
       </c>
       <c r="G42" s="10" t="n">
-        <v>0.000942</v>
+        <v>0.000552</v>
       </c>
       <c r="H42" s="10" t="n">
         <v>0.002515</v>
       </c>
-      <c r="I42" s="5" t="n">
+      <c r="I42" s="6" t="n">
         <v>-0.000496</v>
       </c>
-      <c r="J42" s="5" t="n">
-        <v>-0.000461</v>
+      <c r="J42" s="10" t="n">
+        <v>0.002997</v>
       </c>
       <c r="K42" s="10" t="n">
-        <v>0.000964</v>
-      </c>
-      <c r="L42" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="M42" t="inlineStr"/>
-      <c r="N42" s="10" t="n">
-        <v>0.000552</v>
-      </c>
+        <v>0.000319</v>
+      </c>
+      <c r="L42" s="6" t="n">
+        <v>-0.000684</v>
+      </c>
+      <c r="M42" s="10" t="n">
+        <v>0.000942</v>
+      </c>
+      <c r="N42" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="O42" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>